<commit_message>
Feat: adiciona campos NBM, EAN produto e EAN embalagem
- Adicionados campos nbm, ean_produto e ean_embalagem na migration
- Atualizado Model Product com novos campos no fillable
- ProductImportController agora mapeia NBM e EAN (produto/embalagem)
- Templates Excel/CSV atualizados com os 3 novos campos
- Interface de importação documentada com novos campos
</commit_message>
<xml_diff>
--- a/storage/app/public/modelo_importacao_produtos.xlsx
+++ b/storage/app/public/modelo_importacao_produtos.xlsx
@@ -60,9 +60,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
-    <row r="1" spans="1:11" customHeight="0">
+    <row r="1" spans="1:14" customHeight="0">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>codigo</t>
@@ -118,8 +118,23 @@
           <t>peso_bruto</t>
         </is>
       </c>
+      <c r="L1" s="0" t="inlineStr">
+        <is>
+          <t>nbm</t>
+        </is>
+      </c>
+      <c r="M1" s="0" t="inlineStr">
+        <is>
+          <t>ean_produto</t>
+        </is>
+      </c>
+      <c r="N1" s="0" t="inlineStr">
+        <is>
+          <t>ean_embalagem</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:11" customHeight="0">
+    <row r="2" spans="1:14" customHeight="0">
       <c r="A2" s="0" t="inlineStr">
         <is>
           <t>PROD001</t>
@@ -167,8 +182,23 @@
       <c r="K2" s="0">
         <v>0.494</v>
       </c>
+      <c r="L2" s="0" t="inlineStr">
+        <is>
+          <t>22021000</t>
+        </is>
+      </c>
+      <c r="M2" s="0" t="inlineStr">
+        <is>
+          <t>7891234567890</t>
+        </is>
+      </c>
+      <c r="N2" s="0" t="inlineStr">
+        <is>
+          <t>17891234567897</t>
+        </is>
+      </c>
     </row>
-    <row r="3" spans="1:11" customHeight="0">
+    <row r="3" spans="1:14" customHeight="0">
       <c r="A3" s="0" t="inlineStr">
         <is>
           <t>PROD002</t>
@@ -216,8 +246,23 @@
       <c r="K3" s="0">
         <v>0.494</v>
       </c>
+      <c r="L3" s="0" t="inlineStr">
+        <is>
+          <t>22021000</t>
+        </is>
+      </c>
+      <c r="M3" s="0" t="inlineStr">
+        <is>
+          <t>7899876543210</t>
+        </is>
+      </c>
+      <c r="N3" s="0" t="inlineStr">
+        <is>
+          <t>17899876543217</t>
+        </is>
+      </c>
     </row>
-    <row r="4" spans="1:11" customHeight="0">
+    <row r="4" spans="1:14" customHeight="0">
       <c r="A4" s="0" t="inlineStr">
         <is>
           <t>PROD003</t>
@@ -264,6 +309,21 @@
       </c>
       <c r="K4" s="0">
         <v>0.26</v>
+      </c>
+      <c r="L4" s="0" t="inlineStr">
+        <is>
+          <t>22030000</t>
+        </is>
+      </c>
+      <c r="M4" s="0" t="inlineStr">
+        <is>
+          <t>7895551112222</t>
+        </is>
+      </c>
+      <c r="N4" s="0" t="inlineStr">
+        <is>
+          <t>17895551112229</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>